<commit_message>
Rebrand to the I-CAR Canada design system; replace QR verification with customer notification
- Customer page and letter in I-CAR Blue, Source Sans 3 and the official
  I-CAR Canada, Gold Class and Platinum logos (EN/FR); letter follows the
  letterhead layout
- Remove QR codes and the public verification page; letters carry a reference
- New Notify customers tab: personal links, EN/FR email and phone script,
  contact logging and history, status filters, mail-merge export
- Lists accept contact name, email and phone; notification email wording is
  editable

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RpVGBf7ZaMsjxPtzaka8pX
</commit_message>
<xml_diff>
--- a/samples/SAMPLE-Gold-Class-list.xlsx
+++ b/samples/SAMPLE-Gold-Class-list.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,6 +421,15 @@
       <c r="G1" t="str">
         <v>Gold Class Achieved</v>
       </c>
+      <c r="H1" t="str">
+        <v>Primary Contact</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Phone</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -444,6 +453,15 @@
       <c r="G2" t="str">
         <v>2026-03-15</v>
       </c>
+      <c r="H2" t="str">
+        <v>Jane Doe</v>
+      </c>
+      <c r="I2" t="str">
+        <v>jane@example.com</v>
+      </c>
+      <c r="J2" t="str">
+        <v>905-555-0101</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -467,6 +485,15 @@
       <c r="G3" t="str">
         <v>2026-05-02</v>
       </c>
+      <c r="H3" t="str">
+        <v>Luc Tremblay</v>
+      </c>
+      <c r="I3" t="str">
+        <v>luc@example.com</v>
+      </c>
+      <c r="J3" t="str">
+        <v>450-555-0199</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -490,10 +517,19 @@
       <c r="G4" t="str">
         <v>2026-01-20</v>
       </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v>306-555-0142</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add recognition certificates modelled on the I-CAR plaques, with Scott's letter
- One PDF per request: certificate (page 1) and confirmation letter (page 2), EN or FR
- Gold Class and Gold Class - Aluminum portrait certificates; Platinum landscape
  certificate with technician's role (standard roles translated to French)
- Lists accept an Aluminum column (Gold Class) and a Role column (Platinum)
- Letter adds an Aluminum line for Aluminum shops
- Customer page, emails and phone script now refer to the certificate and letter

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RpVGBf7ZaMsjxPtzaka8pX
</commit_message>
<xml_diff>
--- a/samples/SAMPLE-Gold-Class-list.xlsx
+++ b/samples/SAMPLE-Gold-Class-list.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,12 +422,15 @@
         <v>Gold Class Achieved</v>
       </c>
       <c r="H1" t="str">
+        <v>Aluminum</v>
+      </c>
+      <c r="I1" t="str">
         <v>Primary Contact</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Email</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Phone</v>
       </c>
     </row>
@@ -454,12 +457,15 @@
         <v>2026-03-15</v>
       </c>
       <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
         <v>Jane Doe</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>jane@example.com</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>905-555-0101</v>
       </c>
     </row>
@@ -486,12 +492,15 @@
         <v>2026-05-02</v>
       </c>
       <c r="H3" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="I3" t="str">
         <v>Luc Tremblay</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>luc@example.com</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>450-555-0199</v>
       </c>
     </row>
@@ -524,12 +533,15 @@
         <v/>
       </c>
       <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
         <v>306-555-0142</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>